<commit_message>
feat: expand scoped specialists, weapon systems and media readings
</commit_message>
<xml_diff>
--- a/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Andromeda_Annihilation_Production.xlsx
+++ b/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Andromeda_Annihilation_Production.xlsx
@@ -2,34 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd0b89d107dbb4762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="Rccaf94fdc1ea44a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="R88aba424d5cf4db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="Re71b786de0e24022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R3d6523cec56c4726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="R43b1675d5e814008"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="R313b5b9ee31d4be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="R64394840fe204eaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="R246f94cc3b894d40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R43f242fcbc824a46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="Rc823c3b3d1274da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="R1fbb439cda1f4138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="R3abc3c5b0b1c4ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="R37b9c11d6a1c42b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="R7118fec1436b4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="R7cc967d4037b49dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="Reb9d5e822a6f4f15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="R23293823cb424e93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="R519d4ff3182f44ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R4b907783fa5f4727"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="Rc7d8025586e14347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="R6b1cfc126bcd46d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="Rc59f4a7b631a4ec4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="Ra9bd1199ed1049a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R0ea7002ceff94000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="R1dc6221cac234b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="Re9e5675b1da84522"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R4619fe05930e41b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b4435ae41054f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="R3487a3cabb984ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="Rd445bc60c1a645b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="Rf965f4000e7649f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R6650c1877efe4f53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="R3385cb7dcef0448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="R7692aebc395c4edf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="R399a580e65434adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="Ra1cf7ea4ee4e4547"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R30be9537d6e949de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="R2e6fe4b3d27542ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="Rdb4de4488adf4c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="R7af951be785c43c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="Re39c7d6f4c324bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="Rf54dec1ce0e0424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="R3c60631a2a7140ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="R1696a6a36fdb4afb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="R2cfb700204aa4692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="Re2abd1646ea14ade"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R92b1198f8a764b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="R7f31b7adb7024164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="Rdf5057bf4a5c4f8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="R2daf75b63c914b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="R2590e20ea81f428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R9d99eff9760f4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="Rfb60a30290494969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="R09e0ca2a157d4ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R1e583ae3bb284403"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4228,7 +4228,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7d82969bba54e6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ced8ff74c964f20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4866,7 +4866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R071d44f463c1418c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R922684fc05cc4e25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5504,7 +5504,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2704e4c38fa24cec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfb6a8b7b15c424a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6142,7 +6142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf27290ee1d2a4adf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43823f330fca437f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6902,7 +6902,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ce8b7438e19469d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfa7e3aedb444ee2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7540,7 +7540,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f74f0cc537493a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf612317cefec40b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7819,7 +7819,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f22ae40544945b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf785c76f96c74d65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8147,7 +8147,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66a33d59092e4968"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b70ab027ae84e44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8426,7 +8426,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb647193014714b7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18ce22abc7f84e08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8950,7 +8950,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7cd3ebe69714593"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3af89cedbd04c96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9474,7 +9474,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re819a1af2a704366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fd8d95c045140f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9908,7 +9908,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c90045eebdf409b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2eda4e8bfc54ebd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10648,7 +10648,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d771369deb4aa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red43d976e35041e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11388,7 +11388,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27fa531c9df04445"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e6106eda2f84860"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11822,7 +11822,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28cd8f514d444058"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fb2c62fe0334c4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12297,7 +12297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb3f28217c624c1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe98ecc8da3740c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12919,7 +12919,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f24c2117e60469d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61dca373d75a4ab3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13729,7 +13729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R387c6a9dc433488b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3d0a5cbe5e34ea6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14335,7 +14335,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra740445e7cc54e8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf52591e72a5a4d27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16055,7 +16055,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1a2f577324f40fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8d9e182f4ee4675"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16628,7 +16628,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2caf27a44b545e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f5f99d32cdd4189"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16956,7 +16956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R980f353672c44dd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd72ba105ff94960"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17594,7 +17594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re566eeae6e864bea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41951f86d7884b46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18248,7 +18248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a791fb163df48f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2248a79cbe04427"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18886,7 +18886,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ace8ba00bbe4788"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b272ffe31ad430a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19165,7 +19165,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re395c07dd7b14fb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref5900b9099e4902"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add contextual drones, ammunition modes and partial portraits
</commit_message>
<xml_diff>
--- a/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Andromeda_Annihilation_Production.xlsx
+++ b/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Andromeda_Annihilation_Production.xlsx
@@ -2,34 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b4435ae41054f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="R3487a3cabb984ecf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="Rd445bc60c1a645b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="Rf965f4000e7649f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R6650c1877efe4f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="R3385cb7dcef0448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="R7692aebc395c4edf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="R399a580e65434adc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="Ra1cf7ea4ee4e4547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R30be9537d6e949de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="R2e6fe4b3d27542ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="Rdb4de4488adf4c3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="R7af951be785c43c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="Re39c7d6f4c324bc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="Rf54dec1ce0e0424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="R3c60631a2a7140ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="R1696a6a36fdb4afb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="R2cfb700204aa4692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="Re2abd1646ea14ade"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R92b1198f8a764b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="R7f31b7adb7024164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="Rdf5057bf4a5c4f8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="R2daf75b63c914b0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="R2590e20ea81f428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R9d99eff9760f4121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="Rfb60a30290494969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="R09e0ca2a157d4ac8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R1e583ae3bb284403"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2d9eca9ebc744ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="R1cb10299f6ce404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="Rb72a882637e649d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="Re38540a6600142e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R71dc0216c68b496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="Rcd7ee06eff384e3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="Raddb012fd73d4b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="Rc0be058890b345ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="Rdf1797f97e1e49a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R4af3644dc27646a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="R55f819eb720140bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="R4c6883956bb145f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="R5de53d8ffe9b4068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="Rd1bd5d7285c94c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="R8655b28628ff45bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="Ra765d93ae7c94c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="Rbbc7d9d085a94c73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="R99275b32ef764003"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="Rb92aff1b3d2f4f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R64b9da0dbb2442d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="Rc112b496d07c4f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="Ra84a1b9a79954b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="Ra93bd84fa56b4a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="Rdbde5138e20548e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R3dcdd5d095ee40ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="R5b2c11fb71104cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="Rc20bb44931c74523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R0edb8a1058784d6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4228,7 +4228,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ced8ff74c964f20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d553b09ed1842af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4866,7 +4866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R922684fc05cc4e25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5808629939b44f13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5504,7 +5504,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfb6a8b7b15c424a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac29f65a8a104598"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6142,7 +6142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43823f330fca437f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2909419700a415d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6902,7 +6902,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfa7e3aedb444ee2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfb6cb90d16488e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7540,7 +7540,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf612317cefec40b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f736fe91744d56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7819,7 +7819,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf785c76f96c74d65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb171ac38c16e4e2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8147,7 +8147,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b70ab027ae84e44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e221b7b7dd04a9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8426,7 +8426,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18ce22abc7f84e08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3286ed54f4b4de7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8950,7 +8950,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3af89cedbd04c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a42f7976b4841f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9474,7 +9474,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fd8d95c045140f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1808af263a5f48e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9908,7 +9908,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2eda4e8bfc54ebd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86d21aee910f4ee4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10648,7 +10648,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red43d976e35041e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dc02cc5bf9e4a80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11388,7 +11388,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e6106eda2f84860"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60b121dc04cf43ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11822,7 +11822,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fb2c62fe0334c4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74645f2da8e94bc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12297,7 +12297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe98ecc8da3740c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fb322edb8c24000"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12919,7 +12919,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61dca373d75a4ab3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb15fab7b0ca469a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13729,7 +13729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3d0a5cbe5e34ea6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R729120451e934071"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14335,7 +14335,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf52591e72a5a4d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e7560e666b14a59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16055,7 +16055,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8d9e182f4ee4675"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc66d6e11b5c2498b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16628,7 +16628,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f5f99d32cdd4189"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4bcd589a17e4ddb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16956,7 +16956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd72ba105ff94960"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f895fb7fd2c442e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17594,7 +17594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41951f86d7884b46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea12a7f893f4ccb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18248,7 +18248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2248a79cbe04427"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb16a5cc631ef42bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18886,7 +18886,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b272ffe31ad430a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8a4c5a231974fe2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19165,7 +19165,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref5900b9099e4902"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd63c195618264945"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand scoped arsenal, opponent benches and generated illustrations
</commit_message>
<xml_diff>
--- a/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Andromeda_Annihilation_Production.xlsx
+++ b/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Andromeda_Annihilation_Production.xlsx
@@ -2,34 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2d9eca9ebc744ac8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="R1cb10299f6ce404d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="Rb72a882637e649d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="Re38540a6600142e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R71dc0216c68b496b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="Rcd7ee06eff384e3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="Raddb012fd73d4b01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="Rc0be058890b345ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="Rdf1797f97e1e49a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R4af3644dc27646a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="R55f819eb720140bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="R4c6883956bb145f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="R5de53d8ffe9b4068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="Rd1bd5d7285c94c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="R8655b28628ff45bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="Ra765d93ae7c94c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="Rbbc7d9d085a94c73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="R99275b32ef764003"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="Rb92aff1b3d2f4f0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R64b9da0dbb2442d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="Rc112b496d07c4f48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="Ra84a1b9a79954b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="Ra93bd84fa56b4a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="Rdbde5138e20548e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R3dcdd5d095ee40ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="R5b2c11fb71104cea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="Rc20bb44931c74523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R0edb8a1058784d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7b1617b54fdd4050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="R9729f0cfcf5643d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="Rde3736c65373479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="Rac41d80e7d9943a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R44c2c7cca86940f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="R1f19aa9bdde6436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="R6607db2ab47149f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="Rb73033f6e4004028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="R901d9f98bb2d4797"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R1000e3befb0049f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="Rd5c397fd9a0a4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="R0e328bd0fd3e418b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="Re4a00bcccc294fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="R541dc8f37142432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="R218b3a88dc464b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="Raca5094a75464d02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="R13d382e32373483e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="Rbc8a1f4c338e4065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="R878732cba4024b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="Rb3ece2f51a914c51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="Ra41618c430a84509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="R081357e2634d4607"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="Rc5996229aa0949ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="R74700acad1cb49cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R1b0a90f3ec65486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="Rd09c7670735b4c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="Ra04940ca38144d89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R8263c97977a040d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4228,7 +4228,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d553b09ed1842af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d1980e1bcd4dbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4866,7 +4866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5808629939b44f13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d71d106bdcb495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5504,7 +5504,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac29f65a8a104598"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe257a42887c4836"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6142,7 +6142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2909419700a415d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raefa5b2d10bf4c54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6902,7 +6902,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfb6cb90d16488e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0676d42ab8cb450a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7540,7 +7540,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f736fe91744d56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83eef6079778470f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7819,7 +7819,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb171ac38c16e4e2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42f9dce130174012"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8147,7 +8147,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e221b7b7dd04a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde6234caa9664674"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8426,7 +8426,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3286ed54f4b4de7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0820c48d8d4b9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8950,7 +8950,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a42f7976b4841f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R463fab4a03214fc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9474,7 +9474,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1808af263a5f48e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a07675488ee476d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9908,7 +9908,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86d21aee910f4ee4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb810e8d5ab0e46b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10648,7 +10648,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dc02cc5bf9e4a80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553d6feb03184f3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11388,7 +11388,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60b121dc04cf43ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfecaaca7efb645fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11822,7 +11822,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74645f2da8e94bc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ba7035640e84ac5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12297,7 +12297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fb322edb8c24000"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78efc5a9bb3941b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12919,7 +12919,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb15fab7b0ca469a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6dc4f3a357b4d61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13729,7 +13729,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R729120451e934071"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re50a8ad05d8e40e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14335,7 +14335,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e7560e666b14a59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96a6e9e38b694dd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16055,7 +16055,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc66d6e11b5c2498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9306a3a097f4beb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16628,7 +16628,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4bcd589a17e4ddb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb6e05a4318f4585"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16956,7 +16956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f895fb7fd2c442e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc56c70ad198d4526"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17594,7 +17594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea12a7f893f4ccb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29875849a3484996"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18248,7 +18248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb16a5cc631ef42bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab4c363c25b447aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18886,7 +18886,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8a4c5a231974fe2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re73f4fe2a4a14079"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19165,7 +19165,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd63c195618264945"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c881b3e942241bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>